<commit_message>
argintine spanish, support for manual location, central tibetan, kuansi, zhongjian, uzbek, peras mixtec, pinas mixtec
</commit_message>
<xml_diff>
--- a/IPA_Illustrations_enc.xlsx
+++ b/IPA_Illustrations_enc.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="911">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="950">
   <si>
     <t xml:space="preserve">Language</t>
   </si>
@@ -2752,7 +2752,124 @@
     <t xml:space="preserve">https://doi.org/10.1017/S0025100323000270</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Southern-Tati.zip</t>
+    <t xml:space="preserve">Mexico City Spanish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mexico City, Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100316000232</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Argentine Spanish</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buenos Aires, Argentina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100317000275</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Argentine-Spanish.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Central Tibetan (Lhasa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lhasa, Tibet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100324000033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Central-Tibetan-Lhasa.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ku'ansi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dali Bai Autonomous Prefecture, Yunnan Province, China [lat=26.441270, long=100.364225]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100324000161</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Kuansi.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ykn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zhongjiang Chinese</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zhongjiang county, Dejang region, Sichuan province</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100324000203</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Zhongjiang-Chinese.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cmn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">xina1239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uzbek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uzbekistan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100324000148</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Uzbek.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">uzb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Martín Peras Mixtec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Martín Peras,  Oaxaca, Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100324000124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/San-Martin-Peras-Mixtec.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jmx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Juan Piñas Mixtec</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santiago Juxtlahuaca, Oaxaca, Mexico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S002510032400015X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/San-Juan-Pinas-Mixtec.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vmc</t>
   </si>
 </sst>
 </file>
@@ -2982,8 +3099,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J226"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K234"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.45"/>
@@ -6900,8 +7017,169 @@
       <c r="H226" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="I226" s="10" t="s">
+      <c r="I226" s="1"/>
+    </row>
+    <row r="227" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="0" t="s">
         <v>910</v>
+      </c>
+      <c r="B227" s="0" t="s">
+        <v>911</v>
+      </c>
+      <c r="G227" s="0" t="s">
+        <v>912</v>
+      </c>
+      <c r="H227" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I227" s="0" t="s">
+        <v>913</v>
+      </c>
+      <c r="J227" s="0" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="0" t="s">
+        <v>915</v>
+      </c>
+      <c r="B228" s="0" t="s">
+        <v>916</v>
+      </c>
+      <c r="G228" s="0" t="s">
+        <v>917</v>
+      </c>
+      <c r="H228" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I228" s="0" t="s">
+        <v>918</v>
+      </c>
+      <c r="J228" s="0" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="0" t="s">
+        <v>919</v>
+      </c>
+      <c r="B229" s="0" t="s">
+        <v>920</v>
+      </c>
+      <c r="G229" s="0" t="s">
+        <v>921</v>
+      </c>
+      <c r="H229" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I229" s="10" t="s">
+        <v>922</v>
+      </c>
+      <c r="J229" s="0" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="0" t="s">
+        <v>924</v>
+      </c>
+      <c r="B230" s="0" t="s">
+        <v>925</v>
+      </c>
+      <c r="G230" s="0" t="s">
+        <v>926</v>
+      </c>
+      <c r="H230" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I230" s="10" t="s">
+        <v>927</v>
+      </c>
+      <c r="J230" s="0" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="0" t="s">
+        <v>929</v>
+      </c>
+      <c r="B231" s="0" t="s">
+        <v>930</v>
+      </c>
+      <c r="G231" s="0" t="s">
+        <v>931</v>
+      </c>
+      <c r="H231" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I231" s="10" t="s">
+        <v>932</v>
+      </c>
+      <c r="J231" s="0" t="s">
+        <v>933</v>
+      </c>
+      <c r="K231" s="0" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="0" t="s">
+        <v>935</v>
+      </c>
+      <c r="B232" s="0" t="s">
+        <v>936</v>
+      </c>
+      <c r="G232" s="0" t="s">
+        <v>937</v>
+      </c>
+      <c r="H232" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I232" s="10" t="s">
+        <v>938</v>
+      </c>
+      <c r="J232" s="0" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="0" t="s">
+        <v>940</v>
+      </c>
+      <c r="B233" s="0" t="s">
+        <v>941</v>
+      </c>
+      <c r="G233" s="10" t="s">
+        <v>942</v>
+      </c>
+      <c r="H233" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I233" s="10" t="s">
+        <v>943</v>
+      </c>
+      <c r="J233" s="0" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A234" s="0" t="s">
+        <v>945</v>
+      </c>
+      <c r="B234" s="0" t="s">
+        <v>946</v>
+      </c>
+      <c r="G234" s="10" t="s">
+        <v>947</v>
+      </c>
+      <c r="H234" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I234" s="10" t="s">
+        <v>948</v>
+      </c>
+      <c r="J234" s="0" t="s">
+        <v>949</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed recording link for Mecapalapa Tepehua
</commit_message>
<xml_diff>
--- a/IPA_Illustrations_enc.xlsx
+++ b/IPA_Illustrations_enc.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="950">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="951">
   <si>
     <t xml:space="preserve">Language</t>
   </si>
@@ -2522,6 +2522,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://doi.org/10.1017/S0025100321000098  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Mecapalapa-Tepehua.zip</t>
   </si>
   <si>
     <t xml:space="preserve">Northern Tepehuan</t>
@@ -2976,7 +2979,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3014,10 +3017,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3100,7 +3099,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K234"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.45"/>
@@ -6691,328 +6690,328 @@
         <v>19</v>
       </c>
       <c r="I207" s="7" t="s">
-        <v>822</v>
+        <v>834</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A208" s="2" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B208" s="2" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="G208" s="7" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="H208" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I208" s="7" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A209" s="2" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="B209" s="2" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="G209" s="7" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="H209" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I209" s="7" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A210" s="2" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="B210" s="2" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="G210" s="7" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="H210" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I210" s="7" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="2" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="G211" s="0" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="H211" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I211" s="0" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A212" s="2" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="B212" s="2" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="G212" s="0" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="H212" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I212" s="0" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="2" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="B213" s="2" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="G213" s="0" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="H213" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I213" s="0" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A214" s="2" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="B214" s="2" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="G214" s="0" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="H214" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I214" s="0" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A215" s="2" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="B215" s="2" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="G215" s="7" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="H215" s="2" t="s">
         <v>19</v>
       </c>
       <c r="I215" s="7" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="0" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="B216" s="0" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="G216" s="0" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="H216" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I216" s="1" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A217" s="0" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="B217" s="0" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="G217" s="0" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="H217" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I217" s="1" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="0" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B218" s="0" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="G218" s="0" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="H218" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I218" s="1" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A219" s="0" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="B219" s="0" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="G219" s="0" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="H219" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I219" s="1" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="0" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="B220" s="0" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="G220" s="0" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="H220" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I220" s="1" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="0" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="B221" s="0" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="G221" s="0" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="H221" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I221" s="1" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A222" s="0" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="B222" s="0" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="C222" s="1" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="G222" s="0" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="H222" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I222" s="1" t="s">
-        <v>894</v>
+        <v>895</v>
       </c>
     </row>
     <row r="223" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="0" t="s">
-        <v>895</v>
+        <v>896</v>
       </c>
       <c r="B223" s="2" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="G223" s="7" t="s">
-        <v>897</v>
+        <v>898</v>
       </c>
       <c r="H223" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I223" s="6" t="s">
-        <v>898</v>
+        <v>899</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="0" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="B224" s="0" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="G224" s="0" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="H224" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I224" s="0" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="0" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="B225" s="0" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="G225" s="9" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
       <c r="H225" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I225" s="1" t="s">
-        <v>906</v>
+        <v>907</v>
       </c>
       <c r="J225" s="1"/>
     </row>
     <row r="226" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="0" t="s">
-        <v>907</v>
+        <v>908</v>
       </c>
       <c r="B226" s="0" t="s">
-        <v>908</v>
+        <v>909</v>
       </c>
       <c r="G226" s="0" t="s">
-        <v>909</v>
+        <v>910</v>
       </c>
       <c r="H226" s="0" t="s">
         <v>19</v>
@@ -7021,165 +7020,165 @@
     </row>
     <row r="227" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A227" s="0" t="s">
-        <v>910</v>
+        <v>911</v>
       </c>
       <c r="B227" s="0" t="s">
-        <v>911</v>
+        <v>912</v>
       </c>
       <c r="G227" s="0" t="s">
-        <v>912</v>
+        <v>913</v>
       </c>
       <c r="H227" s="0" t="s">
         <v>19</v>
       </c>
       <c r="I227" s="0" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="J227" s="0" t="s">
-        <v>914</v>
+        <v>915</v>
       </c>
     </row>
     <row r="228" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="0" t="s">
+        <v>916</v>
+      </c>
+      <c r="B228" s="0" t="s">
+        <v>917</v>
+      </c>
+      <c r="G228" s="0" t="s">
+        <v>918</v>
+      </c>
+      <c r="H228" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I228" s="0" t="s">
+        <v>919</v>
+      </c>
+      <c r="J228" s="0" t="s">
         <v>915</v>
-      </c>
-      <c r="B228" s="0" t="s">
-        <v>916</v>
-      </c>
-      <c r="G228" s="0" t="s">
-        <v>917</v>
-      </c>
-      <c r="H228" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="I228" s="0" t="s">
-        <v>918</v>
-      </c>
-      <c r="J228" s="0" t="s">
-        <v>914</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="0" t="s">
-        <v>919</v>
+        <v>920</v>
       </c>
       <c r="B229" s="0" t="s">
-        <v>920</v>
+        <v>921</v>
       </c>
       <c r="G229" s="0" t="s">
-        <v>921</v>
+        <v>922</v>
       </c>
       <c r="H229" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="I229" s="10" t="s">
-        <v>922</v>
+      <c r="I229" s="1" t="s">
+        <v>923</v>
       </c>
       <c r="J229" s="0" t="s">
-        <v>923</v>
+        <v>924</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="0" t="s">
-        <v>924</v>
+        <v>925</v>
       </c>
       <c r="B230" s="0" t="s">
-        <v>925</v>
+        <v>926</v>
       </c>
       <c r="G230" s="0" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="H230" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="I230" s="10" t="s">
-        <v>927</v>
+      <c r="I230" s="1" t="s">
+        <v>928</v>
       </c>
       <c r="J230" s="0" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
     </row>
     <row r="231" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="0" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="B231" s="0" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="G231" s="0" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="H231" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="I231" s="10" t="s">
-        <v>932</v>
+      <c r="I231" s="1" t="s">
+        <v>933</v>
       </c>
       <c r="J231" s="0" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="K231" s="0" t="s">
-        <v>934</v>
+        <v>935</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="0" t="s">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="B232" s="0" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="G232" s="0" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="H232" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="I232" s="10" t="s">
-        <v>938</v>
+      <c r="I232" s="1" t="s">
+        <v>939</v>
       </c>
       <c r="J232" s="0" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="0" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="B233" s="0" t="s">
-        <v>941</v>
-      </c>
-      <c r="G233" s="10" t="s">
         <v>942</v>
       </c>
+      <c r="G233" s="1" t="s">
+        <v>943</v>
+      </c>
       <c r="H233" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="I233" s="10" t="s">
-        <v>943</v>
+      <c r="I233" s="1" t="s">
+        <v>944</v>
       </c>
       <c r="J233" s="0" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
     </row>
     <row r="234" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="0" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="B234" s="0" t="s">
-        <v>946</v>
-      </c>
-      <c r="G234" s="10" t="s">
         <v>947</v>
       </c>
+      <c r="G234" s="1" t="s">
+        <v>948</v>
+      </c>
       <c r="H234" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="I234" s="10" t="s">
-        <v>948</v>
+      <c r="I234" s="1" t="s">
+        <v>949</v>
       </c>
       <c r="J234" s="0" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
     </row>
   </sheetData>
@@ -7206,7 +7205,7 @@
     <hyperlink ref="G206" r:id="rId20" display="https://doi.org/10.1017/S0025100321000177 "/>
     <hyperlink ref="I206" r:id="rId21" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Nafsan.zip"/>
     <hyperlink ref="G207" r:id="rId22" display="https://doi.org/10.1017/S0025100321000098  "/>
-    <hyperlink ref="I207" r:id="rId23" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Mojeno-Trinitario.zip"/>
+    <hyperlink ref="I207" r:id="rId23" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/"/>
     <hyperlink ref="G208" r:id="rId24" display="https://doi.org/10.1017/S002510032100013X  "/>
     <hyperlink ref="I208" r:id="rId25" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Northern-Tepehuan.zip"/>
     <hyperlink ref="G209" r:id="rId26" display="https://doi.org/10.1017/S0025100321000165  "/>

</xml_diff>

<commit_message>
Kam, Gawarbati, Hongshui He Zhuang, Zaiwa
</commit_message>
<xml_diff>
--- a/IPA_Illustrations_enc.xlsx
+++ b/IPA_Illustrations_enc.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1199" uniqueCount="951">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="971">
   <si>
     <t xml:space="preserve">Language</t>
   </si>
@@ -2873,6 +2873,66 @@
   </si>
   <si>
     <t xml:space="preserve">vmc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kam (Rongjiang Variety)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rongjiang County, Qiandongnan Miao and Dong Autonomous Prefecture, Guizhou, China</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100324000215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Kam.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kmc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gawarbati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arandu, Pakistan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100325000076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Gawarbati.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gwt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hongshui He Zhuang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guangxi Zhuang Autonomous Region, China</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S0025100325100704</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Hongshui-He-Zhuang.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zaiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruili County, Dehong Dai and Jingpo Autonomous Prefecture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://doi.org/10.1017/S002510032510073X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Zaiwa.zip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">atb</t>
   </si>
 </sst>
 </file>
@@ -2882,7 +2942,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -2933,6 +2993,28 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Cambria"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2979,7 +3061,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3017,6 +3099,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3098,8 +3196,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K234"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:K238"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.45"/>
@@ -7179,6 +7277,86 @@
       </c>
       <c r="J234" s="0" t="s">
         <v>950</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A235" s="10" t="s">
+        <v>951</v>
+      </c>
+      <c r="B235" s="10" t="s">
+        <v>952</v>
+      </c>
+      <c r="G235" s="10" t="s">
+        <v>953</v>
+      </c>
+      <c r="H235" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="I235" s="11" t="s">
+        <v>954</v>
+      </c>
+      <c r="J235" s="10" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A236" s="10" t="s">
+        <v>956</v>
+      </c>
+      <c r="B236" s="10" t="s">
+        <v>957</v>
+      </c>
+      <c r="G236" s="10" t="s">
+        <v>958</v>
+      </c>
+      <c r="H236" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="I236" s="11" t="s">
+        <v>959</v>
+      </c>
+      <c r="J236" s="10" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A237" s="12" t="s">
+        <v>961</v>
+      </c>
+      <c r="B237" s="12" t="s">
+        <v>962</v>
+      </c>
+      <c r="G237" s="12" t="s">
+        <v>963</v>
+      </c>
+      <c r="H237" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="I237" s="11" t="s">
+        <v>964</v>
+      </c>
+      <c r="J237" s="12" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A238" s="12" t="s">
+        <v>966</v>
+      </c>
+      <c r="B238" s="12" t="s">
+        <v>967</v>
+      </c>
+      <c r="G238" s="13" t="s">
+        <v>968</v>
+      </c>
+      <c r="H238" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="I238" s="11" t="s">
+        <v>969</v>
+      </c>
+      <c r="J238" s="12" t="s">
+        <v>970</v>
       </c>
     </row>
   </sheetData>
@@ -7205,7 +7383,7 @@
     <hyperlink ref="G206" r:id="rId20" display="https://doi.org/10.1017/S0025100321000177 "/>
     <hyperlink ref="I206" r:id="rId21" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Nafsan.zip"/>
     <hyperlink ref="G207" r:id="rId22" display="https://doi.org/10.1017/S0025100321000098  "/>
-    <hyperlink ref="I207" r:id="rId23" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/"/>
+    <hyperlink ref="I207" r:id="rId23" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Mecapalapa-Tepehua.zip"/>
     <hyperlink ref="G208" r:id="rId24" display="https://doi.org/10.1017/S002510032100013X  "/>
     <hyperlink ref="I208" r:id="rId25" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Northern-Tepehuan.zip"/>
     <hyperlink ref="G209" r:id="rId26" display="https://doi.org/10.1017/S0025100321000165  "/>
@@ -7217,6 +7395,11 @@
     <hyperlink ref="G223" r:id="rId32" display="https://doi.org/10.1017/S0025100323000257 "/>
     <hyperlink ref="I223" r:id="rId33" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Tima.zip"/>
     <hyperlink ref="G225" r:id="rId34" display="https://doi.org/10.1017/S0025100323000269"/>
+    <hyperlink ref="I235" r:id="rId35" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Kam.zip"/>
+    <hyperlink ref="I236" r:id="rId36" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Gawarbati.zip"/>
+    <hyperlink ref="I237" r:id="rId37" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Hongshui-He-Zhuang.zip"/>
+    <hyperlink ref="G238" r:id="rId38" display="https://doi.org/10.1017/S002510032510073X"/>
+    <hyperlink ref="I238" r:id="rId39" display="https://www.internationalphoneticassociation.org/sites/default/files/JIPArecordings/Zaiwa.zip"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
added Tai Nuea - removed duplicates that I misunderstood
</commit_message>
<xml_diff>
--- a/IPA_Illustrations_enc.xlsx
+++ b/IPA_Illustrations_enc.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="984">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1236" uniqueCount="982">
   <si>
     <t xml:space="preserve">Language</t>
   </si>
@@ -2953,13 +2953,7 @@
     <t xml:space="preserve">Tai Nuea</t>
   </si>
   <si>
-    <t xml:space="preserve">Mangshi Autonomous Prefecture, Yunnan, China</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dehong Dai Autonomous Prefecture, Yunnan, China</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jingpo Autonomous Prefecture, Yunnan, China</t>
+    <t xml:space="preserve">Mangshi,  Dehong Dai and Jingpo Autonomous Prefecture, Yunnan, China</t>
   </si>
   <si>
     <t xml:space="preserve">https://doi.org/10.1017/S0025100326101108</t>
@@ -3114,7 +3108,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3176,10 +3170,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3262,7 +3252,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K240"/>
-  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="45.45"/>
@@ -7451,26 +7441,22 @@
       <c r="B240" s="15" t="s">
         <v>977</v>
       </c>
-      <c r="C240" s="15" t="s">
+      <c r="C240" s="15"/>
+      <c r="D240" s="15"/>
+      <c r="G240" s="0" t="s">
         <v>978</v>
       </c>
-      <c r="D240" s="15" t="s">
+      <c r="H240" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="I240" s="9" t="s">
         <v>979</v>
       </c>
-      <c r="G240" s="0" t="s">
+      <c r="J240" s="0" t="s">
         <v>980</v>
       </c>
-      <c r="H240" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="I240" s="16" t="s">
+      <c r="K240" s="0" t="s">
         <v>981</v>
-      </c>
-      <c r="J240" s="0" t="s">
-        <v>982</v>
-      </c>
-      <c r="K240" s="0" t="s">
-        <v>983</v>
       </c>
     </row>
   </sheetData>

</xml_diff>